<commit_message>
Added logic for read test data from excel
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/testData.xlsx
+++ b/src/test/resources/TestData/testData.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nikhi\eclipse-workspace\NumpyNinja_Hackathons\Team01_WaitUntilVisible\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F63F0BE7-6280-4117-894C-1A3A2748397A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE1E55E-386E-4375-9158-6598ACA817AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="class_mandatory_data" sheetId="1" r:id="rId1"/>
-    <sheet name="class_all_data" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,22 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
-  <si>
-    <t>classTopic</t>
-  </si>
-  <si>
-    <t>classDescription</t>
-  </si>
-  <si>
-    <t>comments</t>
-  </si>
-  <si>
-    <t>notes</t>
-  </si>
-  <si>
-    <t>recording</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Url</t>
   </si>
@@ -414,24 +398,24 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -442,38 +426,4 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83CFB884-A66A-4FD4-89C2-020487BFDEA8}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="12.81640625" customWidth="1"/>
-    <col min="2" max="2" width="15.6328125" customWidth="1"/>
-    <col min="3" max="3" width="13.81640625" customWidth="1"/>
-    <col min="4" max="4" width="11.54296875" customWidth="1"/>
-    <col min="5" max="5" width="13.08984375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>